<commit_message>
commit pre name change
</commit_message>
<xml_diff>
--- a/bms_sa_review/ami_data_analysis/notebooks/ami_dataset_column_reference.xlsx
+++ b/bms_sa_review/ami_data_analysis/notebooks/ami_dataset_column_reference.xlsx
@@ -8,20 +8,21 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://unsw-my.sharepoint.com/personal/z3553082_ad_unsw_edu_au/Documents/Documents/GitHub/CICCADA/bms_sa_review/ami_data_analysis/notebooks/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="30" documentId="11_0A37DBF18C877FF32CF1DBDEED91CCB9E80CB34E" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E6A8BA2F-740D-4BD9-B0C8-2BFEF20BF3F2}"/>
+  <xr:revisionPtr revIDLastSave="18" documentId="11_FD25D7C65C90A3E4CC61D21805B5FB9F898F4A10" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{840E69BF-5460-441B-A777-BAA74EE498F4}"/>
   <bookViews>
-    <workbookView xWindow="5160" yWindow="2085" windowWidth="28800" windowHeight="18435" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ami_raw" sheetId="1" r:id="rId1"/>
     <sheet name="ami_meter" sheetId="2" r:id="rId2"/>
+    <sheet name="ami_raw_phaseseparate" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="83">
   <si>
     <t>Column</t>
   </si>
@@ -149,6 +150,9 @@
     <t>year-month partition key (Parquet is written partitioned by this).</t>
   </si>
   <si>
+    <t>site_id, device_id, circuit_id</t>
+  </si>
+  <si>
     <t>t_stamp, year, month</t>
   </si>
   <si>
@@ -164,6 +168,9 @@
     <t>S_kva</t>
   </si>
   <si>
+    <t>sqrt(P_kw² + Q_kvar²).</t>
+  </si>
+  <si>
     <t>kVA</t>
   </si>
   <si>
@@ -191,55 +198,79 @@
     <t>energy_export_kwh</t>
   </si>
   <si>
+    <t>Keys. device_id groups the phases belonging to one physical meter. Grain is one row per (site_id, device_id, circuit_id, t_stamp) -- EVERY kept circuit gets a row, load AND PV alike (this is a circuit-preserving table, not load-only).</t>
+  </si>
+  <si>
+    <t>circuit_type</t>
+  </si>
+  <si>
+    <t>ac_load_net or pv_site_net -- tells you which physical thing this row's readings belong to.</t>
+  </si>
+  <si>
+    <t>This circuit's own raw voltage. No polarity correction -- voltage has no sign-convention ambiguity.</t>
+  </si>
+  <si>
+    <t>P_kw_signed</t>
+  </si>
+  <si>
+    <t>Q_kvar_signed</t>
+  </si>
+  <si>
+    <t>Same pattern as P_kw_signed, reactive power. Reasonable-by-construction but not independently validated against real plots the way active power was.</t>
+  </si>
+  <si>
+    <t>n_phases_at_site</t>
+  </si>
+  <si>
+    <t>Number of kept ac_load_net circuits at the site this month -- a per-site topology tag, copied onto every row (load or PV) for that site.</t>
+  </si>
+  <si>
+    <t>pv_allocation_method</t>
+  </si>
+  <si>
+    <t>direct_matched_circuit (kept PV circuit count == kept load circuit count -- a real count match, but not a verified circuit-to-phase label) / equal_split_across_load_phases (counts don't match) / no_pv_present (no surviving PV circuit -- no PV rows for that site). A per-site descriptive tag only -- carries no allocated Watts. This table does NOT split PV across load phases or compute a per-phase gross load for you; do that explicitly from these raw rows if you need it.</t>
+  </si>
+  <si>
     <t>ami_raw: site-level ground truth (one row per site_id, t_stamp)</t>
   </si>
   <si>
-    <t>ami_meter: synthetic smart meter (one row per site_id, device_id, circuit_id, t_stamp)</t>
-  </si>
-  <si>
     <t>UTC</t>
   </si>
   <si>
-    <t>(P_pv_kw / normalization_capacit: PV output as a fraction of site capacity.</t>
+    <t>(P_pv_kw / normalization_capacity): PV output as a fraction of site capacity.</t>
   </si>
   <si>
     <t>(P_load_kw + P_pv_kw): Gross house consumption, PV-independent ("what the house would have consumed without solar"). Derived, not independently measured.</t>
   </si>
   <si>
+    <t>(Q_pv_kvar / normalization_capacity).</t>
+  </si>
+  <si>
     <t>(Q_load_kvar + Q_pv_kvar): Gross reactive load, derived. Reactive-power columns are reasonable-by-construction but not independently validated against real plots the way active power was.</t>
   </si>
   <si>
-    <t>Raw power: Deliberately NOT polarity-corrected. ac_load_net is already net-of-solar as landed, and this table is meant to show what a real meter would report, sign quirks included.</t>
+    <t>ami_meter: Synthetic smart meter (one row per site_id, device_id, circuit_id, t_stamp)</t>
+  </si>
+  <si>
+    <t>ami_raw_phaseseparate: Per-circuit ground truth, load and PV alike (one row per site_id, device_id, circuit_id, t_stamp)</t>
+  </si>
+  <si>
+    <t>Raw power. Deliberately NOT polarity-corrected. ac_load_net is already net-of-solar as landed, and this table is meant to show what a real meter would report, sign quirks included.</t>
+  </si>
+  <si>
+    <t>Keys. device_id groups the phases belonging to one physical meter. Grain is one row per (site_id, device_id, circuit_id, t_stamp), every kept ac_load_net circuit, per phase. PV circuits are deliberately excluded: this table simulates what a real smart meter reports, and a real meter doesn't separately expose PV generation.</t>
   </si>
   <si>
     <t>Raw reactive power. No raw instantaneous field exists in ts for this. It is always derived once, in the interval table, from energy_reactive.</t>
   </si>
   <si>
-    <t>SQRT(P_kw² + Q_kvar²).</t>
-  </si>
-  <si>
     <t>Raw energy_import. The real measured accumulator register (not derived by clipping instantaneous power at zero).</t>
   </si>
   <si>
     <t>Raw energy_export. The real measured accumulator register.</t>
   </si>
   <si>
-    <t>device_id</t>
-  </si>
-  <si>
-    <t>circuit_id</t>
-  </si>
-  <si>
-    <t>Site key</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Device key. Device_id groups the phases belonging to one physical meter. </t>
-  </si>
-  <si>
-    <t>Circuit key. Grain is one row per (site_id, device_id, circuit_id, t_stamp) every kept ac_load_net circuit, per phase. PV circuits are deliberately excluded: this table simulates what a real smart meter reports.</t>
-  </si>
-  <si>
-    <t>(Q_pv_kvar / normalization_capacity)</t>
+    <t>This circuit's own power, polarity-corrected via circuit_polarity. Meaning depends on circuit_type: on a load row, this is ac_load_net's own reading -- already net-of-solar as landed (see ami_raw), NOT a PV-independent gross load figure. On a PV row, this is that PV circuit's own undivided generation reading. NOT the same as ami_meter. P_kw, which is the raw, uncorrected sensor reading.</t>
   </si>
 </sst>
 </file>
@@ -632,7 +663,7 @@
   <sheetData>
     <row r="1" spans="1:4" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>56</v>
+        <v>69</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
@@ -672,7 +703,7 @@
         <v>9</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>58</v>
+        <v>70</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
@@ -686,7 +717,7 @@
         <v>12</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>58</v>
+        <v>70</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
@@ -753,7 +784,7 @@
         <v>14</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>59</v>
+        <v>71</v>
       </c>
       <c r="D11" s="3" t="s">
         <v>25</v>
@@ -767,7 +798,7 @@
         <v>14</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>60</v>
+        <v>72</v>
       </c>
       <c r="D12" s="3" t="s">
         <v>21</v>
@@ -809,7 +840,7 @@
         <v>14</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D15" s="3" t="s">
         <v>25</v>
@@ -823,7 +854,7 @@
         <v>14</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>61</v>
+        <v>74</v>
       </c>
       <c r="D16" s="3" t="s">
         <v>29</v>
@@ -874,7 +905,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:D13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -885,7 +916,7 @@
   <sheetData>
     <row r="1" spans="1:4" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>57</v>
+        <v>75</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
@@ -902,165 +933,278 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" ht="51" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>4</v>
+        <v>42</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>5</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>69</v>
+        <v>78</v>
+      </c>
+      <c r="D4" s="3"/>
+    </row>
+    <row r="5" spans="1:4" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="D5" s="3"/>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="38.25" x14ac:dyDescent="0.25">
+      <c r="A7" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A8" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A10" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A12" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A13" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>56</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <dimension ref="A1:D11"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="22" customWidth="1"/>
+    <col min="2" max="2" width="12" customWidth="1"/>
+    <col min="3" max="3" width="78" customWidth="1"/>
+    <col min="4" max="4" width="16" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="38.25" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>58</v>
       </c>
       <c r="D4" s="3"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>67</v>
+        <v>59</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>5</v>
+        <v>38</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="D5" s="3"/>
     </row>
-    <row r="6" spans="1:4" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>68</v>
+        <v>43</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>5</v>
+        <v>44</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>71</v>
+        <v>45</v>
       </c>
       <c r="D6" s="3"/>
     </row>
     <row r="7" spans="1:4" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>42</v>
+        <v>16</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>43</v>
+        <v>14</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="D7" s="3"/>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+        <v>61</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="63.75" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>16</v>
+        <v>62</v>
       </c>
       <c r="B8" s="3" t="s">
         <v>14</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>45</v>
+        <v>82</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" ht="38.25" x14ac:dyDescent="0.25">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
-        <v>26</v>
+        <v>63</v>
       </c>
       <c r="B9" s="3" t="s">
         <v>14</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>21</v>
+        <v>29</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>33</v>
+        <v>65</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="D10" s="3" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+        <v>66</v>
+      </c>
+      <c r="D10" s="3"/>
+    </row>
+    <row r="11" spans="1:4" ht="76.5" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
-        <v>46</v>
+        <v>67</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>14</v>
+        <v>38</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="D11" s="3" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A12" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="B12" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="C12" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="D12" s="3" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A13" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="B13" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="C13" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="D13" s="3" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A14" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="B14" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="C14" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="D14" s="3" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A15" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="B15" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="C15" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="D15" s="3" t="s">
-        <v>54</v>
-      </c>
+        <v>68</v>
+      </c>
+      <c r="D11" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>